<commit_message>
speeded up parametrization of ue_intercept
</commit_message>
<xml_diff>
--- a/Results/2_parametrization/genetic_algorithm_run_iML1515iML1515final_run_1.xlsx
+++ b/Results/2_parametrization/genetic_algorithm_run_iML1515iML1515final_run_1.xlsx
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>146.5713881584375</v>
+        <v>291.2374572159707</v>
       </c>
     </row>
     <row r="3">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>32.70996287196558</v>
+        <v>81.37133126159945</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>62.74953453296263</v>
+        <v>96.05790266138568</v>
       </c>
     </row>
     <row r="5">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>87.39822738608792</v>
+        <v>61.95360361399488</v>
       </c>
     </row>
     <row r="6">
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>84.63270214502067</v>
+        <v>73.9089207415628</v>
       </c>
     </row>
     <row r="7">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>7.935080699368772</v>
+        <v>74.097785365391</v>
       </c>
     </row>
     <row r="8">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>330.6878306878307</v>
+        <v>347.2016697834046</v>
       </c>
     </row>
     <row r="9">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>30.04957296681992</v>
+        <v>54.15726798036541</v>
       </c>
     </row>
     <row r="10">
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1.005750184280706</v>
+        <v>0.9024303496134286</v>
       </c>
     </row>
     <row r="11">
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1.276449634618044</v>
+        <v>0.9024303496134286</v>
       </c>
     </row>
     <row r="12">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>20.0749437458249</v>
+        <v>19.0735590879787</v>
       </c>
     </row>
     <row r="13">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>19.33131118024431</v>
+        <v>35.61937131874576</v>
       </c>
     </row>
     <row r="14">
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>28.47730927556741</v>
+        <v>5.202424815028913</v>
       </c>
     </row>
     <row r="15">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>12.98384992978067</v>
+        <v>16.91255500973224</v>
       </c>
     </row>
     <row r="16">
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>7.736098772033571</v>
+        <v>33.73714294241403</v>
       </c>
     </row>
     <row r="17">
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>14.22727098758386</v>
+        <v>26.68416205552244</v>
       </c>
     </row>
     <row r="18">
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>7.671209521806778</v>
+        <v>3.539701963527189</v>
       </c>
     </row>
     <row r="19">
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>7.663998062541289</v>
+        <v>11.07198621322935</v>
       </c>
     </row>
     <row r="20">
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>6.758583400919171</v>
+        <v>13.19124598053658</v>
       </c>
     </row>
     <row r="21">
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>11.91681836328804</v>
+        <v>5.928776545222211</v>
       </c>
     </row>
     <row r="22">
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>14.86069398828169</v>
+        <v>0.6456340315989516</v>
       </c>
     </row>
     <row r="23">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6.245757649019942</v>
+        <v>6.758583400919171</v>
       </c>
     </row>
     <row r="24">
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>386.5344889553066</v>
+        <v>141.5970080692576</v>
       </c>
     </row>
     <row r="25">
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>35.94971854462634</v>
+        <v>17.58746487517589</v>
       </c>
     </row>
     <row r="26">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>64.85003358916055</v>
+        <v>55.31496749064262</v>
       </c>
     </row>
     <row r="27">
@@ -1266,7 +1266,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>20.62238161460763</v>
+        <v>3.431684374717887</v>
       </c>
     </row>
     <row r="28">
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>3.270373802268027</v>
+        <v>7.888661404364036</v>
       </c>
     </row>
     <row r="29">
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>4.13509345472191</v>
+        <v>3.646511640874274</v>
       </c>
     </row>
     <row r="30">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>41.139114576167</v>
+        <v>9.180732016005397</v>
       </c>
     </row>
     <row r="31">
@@ -1366,7 +1366,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>22.18365121545629</v>
+        <v>24.52179224668194</v>
       </c>
     </row>
     <row r="32">
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>22.56814677600482</v>
+        <v>29.4625399863953</v>
       </c>
     </row>
     <row r="33">
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>15.77714350853576</v>
+        <v>2.715553724869807</v>
       </c>
     </row>
     <row r="34">
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>271.214389550652</v>
+        <v>82.12121062485519</v>
       </c>
     </row>
     <row r="35">
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>374.8388401603182</v>
+        <v>158.8488980852692</v>
       </c>
     </row>
     <row r="36">
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>34.76166970072938</v>
+        <v>12.77961940100785</v>
       </c>
     </row>
     <row r="37">
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.1460244871004775</v>
+        <v>12.48409878103913</v>
       </c>
     </row>
     <row r="38">
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>10.5263322135823</v>
+        <v>8.036900769243925</v>
       </c>
     </row>
     <row r="39">
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>182.6599676862326</v>
+        <v>274.1344332618728</v>
       </c>
     </row>
     <row r="40">
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>50.98918616000964</v>
+        <v>137.7093307319506</v>
       </c>
     </row>
     <row r="41">
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>188.2123909386367</v>
+        <v>15.01639494216529</v>
       </c>
     </row>
     <row r="42">
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>19.31745099870974</v>
+        <v>10.92414406022295</v>
       </c>
     </row>
     <row r="43">
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>66.21572953757459</v>
+        <v>39.22668042739705</v>
       </c>
     </row>
     <row r="44">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>156.9631845651255</v>
+        <v>45.92430939023539</v>
       </c>
     </row>
     <row r="45">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>6.758583400919171</v>
+        <v>12.34240968861915</v>
       </c>
     </row>
     <row r="46">
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.8018108942654916</v>
+        <v>0.3246938637062174</v>
       </c>
     </row>
     <row r="47">
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>258.744313134248</v>
+        <v>84.50871634678329</v>
       </c>
     </row>
     <row r="48">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>17.34744058016372</v>
+        <v>110.637359559667</v>
       </c>
     </row>
     <row r="49">
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>80.71672487326232</v>
+        <v>245.9087700047672</v>
       </c>
     </row>
     <row r="50">
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>148.9573148370171</v>
+        <v>46.86973478237639</v>
       </c>
     </row>
     <row r="51">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>172.6829403069612</v>
+        <v>38.00094126055599</v>
       </c>
     </row>
     <row r="52">
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>390.1248978813863</v>
+        <v>100.4394904802596</v>
       </c>
     </row>
     <row r="53">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>179.6821910660003</v>
+        <v>36.75916250491174</v>
       </c>
     </row>
     <row r="54">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>361.9458634644033</v>
+        <v>292.568066003213</v>
       </c>
     </row>
     <row r="55">
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>50.34165038556694</v>
+        <v>0.4671032692063819</v>
       </c>
     </row>
     <row r="56">
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>118.0614570570395</v>
+        <v>84.01469248942257</v>
       </c>
     </row>
     <row r="57">
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>150.1239186311641</v>
+        <v>104.4542706169732</v>
       </c>
     </row>
     <row r="58">
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>225.9613392849828</v>
+        <v>182.3765857644132</v>
       </c>
     </row>
     <row r="59">
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>338.9964212458448</v>
+        <v>22.59813859408348</v>
       </c>
     </row>
     <row r="60">
@@ -2091,7 +2091,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>299.3116710893743</v>
+        <v>224.8401133144717</v>
       </c>
     </row>
     <row r="61">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>132.6925886748273</v>
+        <v>241.1899572101107</v>
       </c>
     </row>
     <row r="62">
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>22.31490260870747</v>
+        <v>149.1105748549722</v>
       </c>
     </row>
     <row r="63">
@@ -2166,7 +2166,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>92.57898109969274</v>
+        <v>44.44378878142754</v>
       </c>
     </row>
     <row r="64">
@@ -2191,7 +2191,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>9.894318167387739</v>
+        <v>20.04537805268745</v>
       </c>
     </row>
     <row r="65">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.8820945717427211</v>
+        <v>0.008826656262615917</v>
       </c>
     </row>
     <row r="66">
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>1.665583191856676</v>
+        <v>1.409274863278473</v>
       </c>
     </row>
     <row r="67">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>3.02784003446508</v>
+        <v>13.0960183783199</v>
       </c>
     </row>
   </sheetData>
@@ -2302,11 +2302,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-3.873463070845681</v>
+        <v>-4.669098046462786</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>41.139114576166996,22.18365121545629,22.568146776004824,15.777143508535762,0.8018108942654916,6.7585834009191705,156.96318456512546,66.21572953757459,188.2123909386367,258.744313134248,50.98918616000964,182.65996768623262,10.526332213582297,0.14602448710047747,34.76166970072938,374.83884016031817,19.31745099870974,80.71672487326232,0.8820945717427211,9.89431816738774,92.57898109969274,22.31490260870747,132.69258867482728,299.31167108937433,338.9964212458448,148.95731483701712,150.12391863116414,179.6821910660003,17.34744058016372,271.214389550652,172.6829403069612,390.1248978813863,225.96133928498278,361.94586346440326,50.341650385566936,118.06145705703953,30.04957296681992,146.57138815843746,330.6878306878307,32.70996287196558,62.749534532962635,87.39822738608792,84.63270214502067,7.935080699368772,1.6655831918566764,3.02784003446508,1.0057501842807062,1.2764496346180436,14.860693988281689,7.663998062541289,6.7585834009191705,7.671209521806778,6.245757649019942,11.91681836328804,386.53448895530664,35.94971854462634,64.85003358916055,20.622381614607633,12.983849929780673,28.477309275567407,19.331311180244313,20.074943745824903,14.227270987583863,7.7360987720335705,4.13509345472191,3.2703738022680273</t>
+          <t>9.180732016005397,24.52179224668194,29.462539986395296,2.7155537248698067,0.32469386370621744,12.342409688619151,45.924309390235386,39.22668042739705,15.016394942165292,84.50871634678329,137.70933073195064,274.1344332618728,8.036900769243925,12.484098781039126,12.779619401007846,158.84889808526924,10.924144060222952,245.9087700047672,0.008826656262615917,20.04537805268745,44.44378878142754,149.11057485497216,241.1899572101107,224.8401133144717,22.598138594083483,46.86973478237639,104.45427061697319,36.759162504911735,110.637359559667,82.1212106248552,38.00094126055599,100.43949048025961,182.37658576441322,292.568066003213,0.4671032692063819,84.01469248942257,54.15726798036541,291.2374572159707,347.20166978340455,81.37133126159945,96.05790266138568,61.95360361399488,73.9089207415628,74.097785365391,1.4092748632784726,13.0960183783199,0.9024303496134286,0.9024303496134286,0.6456340315989516,11.071986213229353,13.191245980536584,3.539701963527189,6.7585834009191705,5.928776545222211,141.59700806925756,17.587464875175886,55.314967490642616,3.431684374717887,16.912555009732245,5.2024248150289125,35.619371318745756,19.073559087978698,26.68416205552244,33.73714294241403,3.6465116408742744,7.888661404364036</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2315,11 +2315,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-4.043112753774289</v>
+        <v>-4.719892492815229</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>41.139114576166996,25.420066600574494,22.568146776004824,14.317632841559982,0.9348839552646018,6.7585834009191705,8.675695431748764,155.1569676959511,131.38381587159637,342.67668720368,50.98918616000964,182.37658576441322,10.526332213582297,0.12625729277925216,28.06987080774354,195.8888233130593,56.73171973377721,80.71672487326232,0.8820945717427211,6.7585834009191705,92.57898109969274,22.31490260870747,86.11233646813679,199.9791685748329,253.92811409234372,148.95731483701712,80.90064933627582,179.6821910660003,66.21572953757459,271.214389550652,172.6829403069612,390.1248978813863,182.37658576441322,273.37641745672454,33.92059290786593,134.76896990582912,30.04957296681992,146.57138815843746,330.6878306878307,32.70996287196558,62.749534532962635,87.39822738608792,84.63270214502067,7.935080699368772,2.3013334388701154,9.03532528149454,1.0057501842807062,1.321124927121248,7.596578225447472,7.663998062541289,6.7585834009191705,7.671209521806778,6.245757649019942,11.441791404815692,281.12800139592343,35.94971854462634,64.85003358916055,16.15227925406432,10.704840986010058,28.477309275567407,19.331311180244313,19.073559087978698,14.227270987583863,7.7360987720335705,4.13509345472191,12.897069767198998</t>
+          <t>24.809118641174802,45.78216022758797,22.568146776004824,24.255407500548177,11.136171283810416,10.94988802279714,55.812771901662565,130.2462617600637,46.89894777520771,223.62782635592004,48.39924342302681,354.56798323374346,6.7585834009191705,8.138007929389591,11.262284033237288,43.31592510903568,42.4697700177014,204.74860970967217,4.2623202046867785,10.335605055744553,12.533849908230781,505.1156329008741,44.849922811935805,70.69520891598323,195.34583976960107,36.747954200215865,99.02162000702762,275.6314791285956,57.27634900061284,343.5429459382562,2.8405694074260817,416.4640860697068,43.01450359942585,11.35035758605274,44.92387200649778,120.63807436421091,44.84337107351443,315.51453012329057,88.01045845131537,44.23470838303909,2.7163820332883803,32.44722737759192,84.41863003022884,107.00291130470463,2.160829291034198,11.193203901931001,0.9024303496134286,0.43499969488111073,4.929884228570731,14.958413270980516,1.6830506260644438,6.7585834009191705,2.542728865910718,2.035947340992194,131.7185123063304,33.58089166670025,69.07409265598756,3.431684374717887,12.05943206792191,24.10754632382966,20.321480444909508,19.073559087978698,16.221354676447707,0.7905641559716957,6.7585834009191705,6.7585834009191705</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -2328,11 +2328,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>-4.077019286934247</v>
+        <v>-4.807678740843243</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>41.139114576166996,25.420066600574494,22.568146776004824,22.03523639599113,1.6549118058498,6.7585834009191705,8.675695431748764,155.1569676959511,66.9075121505496,172.6829403069612,50.98918616000964,182.37658576441322,6.7585834009191705,1.0439624712780842,43.816294052902045,139.2605605822254,42.4697700177014,100.40402579981847,5.898098507467123,6.7585834009191705,92.57898109969274,273.45715473299646,86.11233646813679,234.76823679663434,208.90802810730577,246.3224064713823,123.09570937595399,266.2236704789896,66.21572953757459,271.214389550652,172.6829403069612,390.1248978813863,182.37658576441322,273.37641745672454,33.92059290786593,84.01469248942257,44.91304997786726,188.81034378587395,330.6878306878307,32.70996287196558,34.944556965917876,87.39822738608792,84.63270214502067,74.097785365391,2.3013334388701154,6.7585834009191705,0.9024303496134286,1.321124927121248,7.596578225447472,7.663998062541289,6.7585834009191705,6.7585834009191705,6.7585834009191705,10.115668078543084,281.12800139592343,33.58089166670025,64.85003358916055,33.58089166670025,2.8044936485904457,15.230798380174132,15.280591927511557,25.253077341722808,14.859258362121578,6.777042917235754,4.891504517858715,6.7585834009191705</t>
+          <t>24.809118641174802,45.78216022758797,22.568146776004824,24.255407500548177,11.136171283810416,10.94988802279714,55.812771901662565,130.2462617600637,46.89894777520771,223.62782635592004,48.39924342302681,354.56798323374346,6.7585834009191705,8.138007929389591,11.262284033237288,43.31592510903568,42.4697700177014,204.74860970967217,4.2623202046867785,10.335605055744553,12.533849908230781,505.1156329008741,44.849922811935805,70.69520891598323,25.02115430502808,196.46788252107086,123.09570937595399,54.44163405917775,424.11547270563705,56.55262339459598,453.29473090296636,35.665393582612786,182.37658576441322,239.03180078010345,87.68136913946489,84.01469248942257,44.84337107351443,179.42460800523105,347.20166978340455,55.600618605499,52.39596207062338,32.44722737759192,84.41863003022884,107.00291130470463,2.160829291034198,11.193203901931001,0.9024303496134286,0.43499969488111073,4.929884228570731,14.958413270980516,1.6830506260644438,6.7585834009191705,2.542728865910718,2.035947340992194,131.7185123063304,33.58089166670025,69.07409265598756,3.431684374717887,12.05943206792191,24.10754632382966,20.321480444909508,19.073559087978698,16.221354676447707,0.7905641559716957,6.7585834009191705,6.7585834009191705</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2341,11 +2341,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-4.420856047839238</v>
+        <v>-4.926274500848887</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35.25330351162232,15.552719376716581,22.568146776004824,32.11375909136936,10.030433241391549,6.7585834009191705,40.23100335884485,286.23012442997924,69.39642880541969,117.2297562321697,48.39924342302681,131.99450836057588,3.3815248528713955,6.530034469516218,43.816294052902045,94.65252955794274,83.08086052106502,101.3602816009449,6.7585834009191705,6.7585834009191705,87.50271656084925,273.45715473299646,100.40402579981847,322.79253572227526,106.08683844247548,246.3224064713823,149.62307393299318,266.2236704789896,176.27698725509674,425.0746203728048,172.6829403069612,62.65835628817881,195.49859095923722,187.3146523296262,50.278134273436756,128.8610439634523,1.8628999543045912,67.36286394800425,330.6878306878307,21.95504100702457,70.86239075293061,12.385688553707633,92.83487142405318,15.301096435025904,9.359244388057945,3.204343450739568,1.3000479715091129,1.1846234482868918,3.4946689649399003,8.44525059553626,13.044659084649393,6.7585834009191705,2.794529062832736,1.6398829151436713,210.5812885890211,33.58089166670025,69.48787507935415,21.981924949136197,19.642264001414386,0.6639520697185533,39.47846481989109,29.894010793135347,10.012283068868888,3.3742735709123157,0.9035376860608766,13.116344422303685</t>
+          <t>1.6353880924470472,25.420066600574494,25.608688746639718,22.9231990380021,7.470316122704257,0.4702203327834232,5.972299371306654,112.31736365144323,51.83778092541572,209.83159723537216,48.39924342302681,182.37658576441322,6.7585834009191705,6.7585834009191705,11.262284033237288,79.43802541479826,42.4697700177014,122.00358104273103,4.2623202046867785,6.7585834009191705,84.01469248942257,505.1156329008741,30.40141109013832,438.85185761568505,106.08683844247548,37.54137512996623,123.09570937595399,92.1174102840359,253.7993675764115,367.41794619167376,141.58640595754062,272.33115468409585,182.37658576441322,165.45714768643563,63.47410302257665,84.01469248942257,71.21115950704504,39.37003594395405,672.7681199951508,28.282046669902133,68.6986697560264,70.5736224028907,66.31649424338706,121.97931473345784,3.2135581304395866,6.7585834009191705,0.9024303496134286,0.3395142980885454,4.929884228570731,7.663998062541289,1.6830506260644438,6.7585834009191705,2.542728865910718,2.035947340992194,131.7185123063304,33.58089166670025,69.07409265598756,3.431684374717887,12.05943206792191,24.10754632382966,20.321480444909508,19.073559087978698,16.221354676447707,0.7905641559716957,6.7585834009191705,6.7585834009191705</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -2354,11 +2354,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-4.527916830806915</v>
+        <v>-4.932397913497547</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>24.809118641174802,25.420066600574494,14.663897116713407,13.702235503131847,0.7356238413231273,6.7585834009191705,45.924309390235386,223.9482840567913,8.601358168914638,172.6829403069612,23.16533772397172,182.37658576441322,9.265174266680896,7.763821119126628,35.59169087329396,24.763392953230277,17.5603376574665,27.13302081725416,18.94111536757602,9.359244388057945,39.83259711018245,393.9444406513736,100.40402579981847,234.76823679663434,67.96201992543956,200.0860897936813,123.09570937595399,374.4796181358267,200.36691294926464,218.03445717083338,333.2932291303555,16.840438998514383,14.882462129817508,273.37641745672454,16.142279082727445,102.12002196932902,27.1179071325236,246.7354692461067,223.1909501884104,29.697438964990603,42.89993344700622,54.78552496409889,1.9280457690183903,74.097785365391,6.7585834009191705,11.13225328286807,0.9024303496134286,0.7068104255253372,0.07057866421903752,7.663998062541289,13.116344422303685,9.652517176718659,7.25850359516681,11.192293764493465,210.5812885890211,33.58089166670025,48.27471334889656,37.425589682973175,12.1503387958695,14.07512045656131,15.619005940052043,19.073559087978698,14.922860713204354,5.763719946688966,6.7585834009191705,12.317787210325907</t>
+          <t>1.6353880924470472,25.420066600574494,25.608688746639718,22.9231990380021,7.470316122704257,0.4702203327834232,5.972299371306654,112.31736365144323,51.83778092541572,209.83159723537216,48.39924342302681,182.37658576441322,4.2623202046867785,12.484098781039126,11.262284033237288,79.43802541479826,12.859453860804312,122.00358104273103,4.2623202046867785,12.633808222162502,84.01469248942257,376.4545776189341,30.40141109013832,438.85185761568505,106.08683844247548,21.59362246674353,107.55280388310864,92.1174102840359,273.28243382361376,367.41794619167376,110.30216459932073,330.42204224748264,182.37658576441322,165.45714768643563,63.47410302257665,84.01469248942257,71.21115950704504,39.37003594395405,672.7681199951508,28.282046669902133,68.6986697560264,70.5736224028907,66.31649424338706,5.155889133494859,6.7585834009191705,26.331781296890263,0.9024303496134286,1.4855752448970638,4.684820373112696,15.705404260543892,1.6830506260644438,6.7585834009191705,2.542728865910718,2.035947340992194,131.7185123063304,66.01779467324673,69.07409265598756,3.431684374717887,18.08194465994709,21.16299713972718,38.7873728022904,19.073559087978698,16.221354676447707,0.7905641559716957,6.7585834009191705,6.7585834009191705</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -2367,11 +2367,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>-4.78103548086755</v>
+        <v>-4.941700003214792</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>16.119992789896514,25.420066600574494,12.749077169166302,2.6400289794432967,6.991123807205158,6.7585834009191705,45.924309390235386,149.99610010139736,92.0937353821321,172.6829403069612,96.0447648730402,284.04717613960486,0.8173861290034279,6.7585834009191705,28.06987080774354,106.08683844247548,59.73947857427783,100.40402579981847,6.7585834009191705,6.7585834009191705,84.01469248942257,273.45715473299646,100.40402579981847,234.76823679663434,106.08683844247548,246.3224064713823,123.09570937595399,266.2236704789896,149.99610010139736,271.214389550652,172.6829403069612,272.33115468409585,182.37658576441322,273.37641745672454,44.92387200649778,84.01469248942257,44.84337107351443,188.81034378587395,330.6878306878307,28.282046669902133,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,6.7585834009191705,6.7585834009191705,0.9024303496134286,0.9024303496134286,4.929884228570731,7.663998062541289,6.7585834009191705,6.7585834009191705,7.532377987800143,6.7585834009191705,239.01653502104344,31.03285090181452,34.94719478867431,37.98321125750463,11.459970281064813,7.325955223007839,12.333181388538627,35.66219101430774,15.693481959883021,10.992854762432373,6.7585834009191705,6.7585834009191705</t>
+          <t>23.505803652187648,25.420066600574494,25.608688746639718,45.30718958122842,6.7585834009191705,0.4702203327834232,23.235431165903087,149.99610010139736,51.83778092541572,172.6829403069612,48.39924342302681,182.37658576441322,4.2623202046867785,12.484098781039126,11.262284033237288,79.43802541479826,12.859453860804312,122.00358104273103,4.2623202046867785,12.633808222162502,84.01469248942257,376.4545776189341,30.40141109013832,438.85185761568505,106.08683844247548,183.5801377869078,123.09570937595399,54.44163405917775,253.7993675764115,271.214389550652,233.9360067695588,272.33115468409585,257.6846045692983,165.45714768643563,63.47410302257665,84.01469248942257,44.84337107351443,179.42460800523105,347.20166978340455,55.600618605499,52.39596207062338,61.95360361399488,84.41863003022884,8.518812996765039,6.7585834009191705,18.636349571790625,0.9024303496134286,1.4855752448970638,4.929884228570731,14.958413270980516,1.6303994254477026,6.7585834009191705,6.7585834009191705,8.439723229292037,131.7185123063304,33.58089166670025,55.314967490642616,3.431684374717887,19.27967982669594,15.230798380174132,20.321480444909508,19.073559087978698,16.221354676447707,7.7360987720335705,6.7585834009191705,6.7585834009191705</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -2380,11 +2380,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-4.781035480867562</v>
+        <v>-5.011205992972211</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>16.119992789896514,25.420066600574494,12.749077169166302,2.6400289794432967,6.991123807205158,6.7585834009191705,45.924309390235386,149.99610010139736,92.0937353821321,172.6829403069612,96.0447648730402,284.04717613960486,0.8173861290034279,6.7585834009191705,28.06987080774354,106.08683844247548,59.73947857427783,100.40402579981847,6.7585834009191705,6.7585834009191705,84.01469248942257,273.45715473299646,100.40402579981847,234.76823679663434,106.08683844247548,246.3224064713823,123.09570937595399,266.2236704789896,149.99610010139736,271.214389550652,172.6829403069612,272.33115468409585,182.37658576441322,273.37641745672454,44.92387200649778,84.01469248942257,44.84337107351443,188.81034378587395,330.6878306878307,28.282046669902133,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,6.7585834009191705,6.7585834009191705,0.9024303496134286,0.9024303496134286,4.929884228570731,7.663998062541289,6.7585834009191705,6.7585834009191705,7.532377987800143,6.7585834009191705,239.01653502104344,31.03285090181452,34.94719478867431,37.98321125750463,11.459970281064813,7.325955223007839,12.333181388538627,35.66219101430774,15.693481959883021,10.992854762432373,6.7585834009191705,6.7585834009191705</t>
+          <t>42.87319408525826,75.91466713154222,20.619269267637463,28.31106544763118,4.113718371674152,24.328596140738114,52.04949803851795,170.0019406208649,84.09080372487385,172.6829403069612,90.4137700678956,182.37658576441322,12.118282758687485,6.7585834009191705,81.85244345868402,106.08683844247548,42.4697700177014,101.96836736106637,0.45498780184301924,6.7585834009191705,132.31995438058453,539.9257819193649,6.7591985309578835,234.76823679663434,106.08683844247548,651.0620815660508,299.18622693415927,320.5598293060303,30.409390488507235,407.462092322603,38.00094126055599,100.43949048025961,182.37658576441322,490.99300403833905,0.714320534996684,84.01469248942257,8.079528094341278,429.6503684435167,55.931162544630695,19.1918683353547,96.05790266138568,66.3028880102485,123.50667835306578,74.097785365391,1.4092748632784726,13.0960183783199,0.9024303496134286,0.18817144542402883,0.6456340315989516,21.454042412680185,13.191245980536584,3.539701963527189,0.8851265560648433,8.565155110210368,276.3657489667987,17.587464875175886,57.87767256329671,43.02522076711055,6.772874593521949,15.230798380174132,21.662036631854583,9.955876853535026,8.734854729309959,4.9285602738116765,11.193203901931001,7.66914804304478</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -2393,11 +2393,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-4.78103548086758</v>
+        <v>-5.011205992972223</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>16.119992789896514,25.420066600574494,12.749077169166302,2.6400289794432967,6.991123807205158,6.7585834009191705,45.924309390235386,149.99610010139736,92.0937353821321,172.6829403069612,96.0447648730402,284.04717613960486,0.8173861290034279,6.7585834009191705,28.06987080774354,106.08683844247548,59.73947857427783,100.40402579981847,6.7585834009191705,6.7585834009191705,84.01469248942257,273.45715473299646,100.40402579981847,234.76823679663434,106.08683844247548,246.3224064713823,123.09570937595399,266.2236704789896,149.99610010139736,271.214389550652,172.6829403069612,272.33115468409585,182.37658576441322,273.37641745672454,44.92387200649778,84.01469248942257,44.84337107351443,188.81034378587395,330.6878306878307,28.282046669902133,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,6.7585834009191705,6.7585834009191705,0.9024303496134286,0.9024303496134286,4.929884228570731,7.663998062541289,6.7585834009191705,6.7585834009191705,7.532377987800143,6.7585834009191705,239.01653502104344,31.03285090181452,34.94719478867431,37.98321125750463,11.459970281064813,7.325955223007839,12.333181388538627,35.66219101430774,15.693481959883021,10.992854762432373,6.7585834009191705,6.7585834009191705</t>
+          <t>42.87319408525826,75.91466713154222,20.619269267637463,28.31106544763118,4.113718371674152,24.328596140738114,52.04949803851795,170.0019406208649,84.09080372487385,172.6829403069612,90.4137700678956,182.37658576441322,12.118282758687485,6.7585834009191705,81.85244345868402,106.08683844247548,42.4697700177014,101.96836736106637,0.45498780184301924,6.7585834009191705,132.31995438058453,539.9257819193649,6.7591985309578835,234.76823679663434,106.08683844247548,651.0620815660508,299.18622693415927,320.5598293060303,30.409390488507235,407.462092322603,38.00094126055599,100.43949048025961,182.37658576441322,490.99300403833905,0.714320534996684,84.01469248942257,8.079528094341278,429.6503684435167,55.931162544630695,19.1918683353547,96.05790266138568,66.3028880102485,123.50667835306578,74.097785365391,1.4092748632784726,13.0960183783199,0.9024303496134286,0.18817144542402883,0.6456340315989516,21.454042412680185,13.191245980536584,3.539701963527189,0.8851265560648433,8.565155110210368,276.3657489667987,17.587464875175886,57.87767256329671,43.02522076711055,6.772874593521949,15.230798380174132,21.662036631854583,9.955876853535026,8.734854729309959,4.9285602738116765,11.193203901931001,7.66914804304478</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -2406,11 +2406,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-4.781035480867607</v>
+        <v>-5.01120599297224</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>16.119992789896514,25.420066600574494,12.749077169166302,2.6400289794432967,6.991123807205158,6.7585834009191705,45.924309390235386,149.99610010139736,92.0937353821321,172.6829403069612,96.0447648730402,284.04717613960486,0.8173861290034279,6.7585834009191705,28.06987080774354,106.08683844247548,59.73947857427783,100.40402579981847,6.7585834009191705,6.7585834009191705,84.01469248942257,273.45715473299646,100.40402579981847,234.76823679663434,106.08683844247548,246.3224064713823,123.09570937595399,266.2236704789896,149.99610010139736,271.214389550652,172.6829403069612,272.33115468409585,182.37658576441322,273.37641745672454,44.92387200649778,84.01469248942257,44.84337107351443,188.81034378587395,330.6878306878307,28.282046669902133,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,6.7585834009191705,6.7585834009191705,0.9024303496134286,0.9024303496134286,4.929884228570731,7.663998062541289,6.7585834009191705,6.7585834009191705,6.7585834009191705,6.7585834009191705,239.01653502104344,31.03285090181452,34.94719478867431,37.98321125750463,11.459970281064813,7.325955223007839,12.333181388538627,35.66219101430774,15.693481959883021,10.992854762432373,6.7585834009191705,6.7585834009191705</t>
+          <t>42.87319408525826,75.91466713154222,20.619269267637463,28.31106544763118,4.113718371674152,24.328596140738114,52.04949803851795,170.0019406208649,84.09080372487385,172.6829403069612,90.4137700678956,182.37658576441322,12.118282758687485,6.7585834009191705,81.85244345868402,106.08683844247548,42.4697700177014,101.96836736106637,0.45498780184301924,6.7585834009191705,132.31995438058453,539.9257819193649,6.7591985309578835,234.76823679663434,106.08683844247548,651.0620815660508,299.18622693415927,320.5598293060303,30.409390488507235,407.462092322603,38.00094126055599,100.43949048025961,182.37658576441322,490.99300403833905,0.714320534996684,84.01469248942257,8.079528094341278,429.6503684435167,55.931162544630695,19.1918683353547,96.05790266138568,66.3028880102485,123.50667835306578,74.097785365391,1.4092748632784726,13.0960183783199,0.9024303496134286,0.18817144542402883,0.6456340315989516,21.454042412680185,13.191245980536584,3.539701963527189,0.8851265560648433,8.565155110210368,276.3657489667987,17.587464875175886,57.87767256329671,43.02522076711055,6.772874593521949,15.230798380174132,21.662036631854583,9.955876853535026,8.734854729309959,4.9285602738116765,11.193203901931001,7.66914804304478</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -2419,11 +2419,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>-4.79314724208921</v>
+        <v>-5.554320441048052</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16.119992789896514,25.420066600574494,12.749077169166302,2.6400289794432967,6.991123807205158,6.7585834009191705,45.924309390235386,149.99610010139736,92.0937353821321,172.6829403069612,96.0447648730402,284.04717613960486,0.8173861290034279,6.7585834009191705,28.06987080774354,106.08683844247548,59.73947857427783,100.40402579981847,6.7585834009191705,6.7585834009191705,101.98771583378617,273.45715473299646,100.40402579981847,371.0792461438465,106.08683844247548,295.9562356420613,123.09570937595399,266.2236704789896,211.17543159708532,509.80776685649283,325.35940928281923,245.82433813168643,182.37658576441322,273.37641745672454,44.92387200649778,125.57407714946986,44.84337107351443,181.48397188037686,641.4516829066745,28.282046669902133,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,6.7585834009191705,6.7585834009191705,0.9024303496134286,0.9024303496134286,4.929884228570731,7.663998062541289,6.7585834009191705,6.7585834009191705,7.532377987800143,6.7585834009191705,239.01653502104344,31.03285090181452,34.94719478867431,37.98321125750463,11.459970281064813,7.325955223007839,12.333181388538627,35.66219101430774,15.693481959883021,10.992854762432373,6.7585834009191705,6.7585834009191705</t>
+          <t>17.389174675184137,4.9063955774777,26.48855346002949,18.92334968531565,1.382077781185087,11.336835025172038,55.812771901662565,130.2462617600637,46.89894777520771,223.62782635592004,48.39924342302681,354.56798323374346,2.580780309348783,8.138007929389591,14.265755740991517,79.43802541479826,1.2892534299059368,122.00358104273103,4.2623202046867785,5.322818482050563,146.6139701727804,326.88717522778535,39.37042922801291,1052.9992210637038,106.08683844247548,100.4445711654097,123.09570937595399,54.44163405917775,150.6441088201207,271.214389550652,417.06545880958635,67.68415631495361,154.5141929661188,24.760979680039455,0.36949305938732846,68.682051554496,15.171690420442474,395.7726062583071,81.88939063656439,87.0837844638941,562.7628718343384,14.432012443431422,163.08722007994322,17.450292522873017,0.07488990408856595,1.7150981141680843,0.8100695501189892,0.31418175704823514,1.3650493795921412,20.298353764457097,9.795469462729097,0.4732257238485097,5.169457708419965,13.451420135540577,19.939645702442927,33.58089166670025,57.87767256329671,43.02522076711055,3.2813437396729683,17.82076007970865,62.40660588929557,9.955876853535026,18.77538344162498,8.045943045439513,28.55181945844303,3.2158823975417508</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -2432,11 +2432,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>-4.853126386208754</v>
+        <v>-6.003364172906589</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15.86484533359101,36.34214052692148,15.320901650504386,24.255407500548177,10.090750054617324,13.221378985987304,42.67560099878069,206.23582713245645,46.89894777520771,220.47250653164585,59.26230254329684,221.39188816311938,6.7585834009191705,6.7585834009191705,43.816294052902045,27.79302046614106,42.4697700177014,100.40402579981847,6.7585834009191705,6.7585834009191705,104.09270661009509,273.45715473299646,132.93327256060874,348.42022162034516,106.08683844247548,246.3224064713823,123.09570937595399,266.2236704789896,131.40085691252713,271.214389550652,124.97876145965007,91.26126034149975,182.37658576441322,264.1318932163335,44.92387200649778,164.35250168589604,30.266111029036672,324.12758763932663,14.45158423912577,41.749971374458404,91.52729721561033,40.59357712860112,47.24981040146311,79.92496037846938,10.59273543031209,1.2179580860554593,0.9214389793747422,0.9024303496134286,5.853591988159366,16.094491571751337,8.90584614047615,6.7585834009191705,6.7585834009191705,8.304244844053969,80.81489324721875,61.202511435630825,34.94719478867431,6.0515815395349755,11.436075434177653,17.53430830775565,20.42389373082748,26.347482339664527,8.606200576779365,12.828196694865065,6.139949738544274,1.6549118058498</t>
+          <t>42.87319408525826,25.420066600574494,22.568146776004824,22.087453753035252,12.953658584125526,11.726112147272802,45.924309390235386,180.4172861299534,23.15001315007426,330.9681510677352,104.76583662285518,153.80584123355416,9.063702493743007,3.336136566583331,81.85244345868402,109.83573377741241,37.10724661997721,4.245129634960418,4.435001074318475,27.165038374638538,84.01469248942257,531.6425430826094,145.60656180637156,33.44683562043491,27.58766110688072,272.38989471817723,256.8830396197169,68.40576367332817,260.8465823177948,691.8669935886252,73.53350486178549,511.95453517620047,138.4715366811512,434.9009687256463,53.62025568201951,92.44098667432446,70.41194768083115,87.30716324463809,68.95380581041096,82.7753223714027,7.958558548987063,70.5736224028907,119.94573605394311,270.21471289537845,0.3255534961953752,7.452826714492409,0.7843380680877265,1.6940455249024926,1.2063130800004742,11.071986213229353,4.881483137555746,5.251983359540708,6.7585834009191705,4.406717420513752,141.59700806925756,7.202682492570821,57.87767256329671,43.02522076711055,1.7288752706917805,15.230798380174132,39.77685154404924,2.0850120946706783,3.1882242796977875,7.329692819782498,6.7585834009191705,6.000288793351045</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -2445,11 +2445,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>-4.853126386208777</v>
+        <v>-6.3177867125755</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15.86484533359101,36.34214052692148,15.320901650504386,24.255407500548177,10.090750054617324,13.221378985987304,42.67560099878069,206.23582713245645,46.89894777520771,220.47250653164585,59.26230254329684,221.39188816311938,11.243605586920193,1.713807437951852,43.816294052902045,127.46327793062652,66.14565238330309,12.14290822744194,0.8900074955439067,13.384452743650984,84.01469248942257,308.8122947381376,216.80270160365524,467.7434254093612,146.90839610035954,246.3224064713823,123.09570937595399,126.2205442068202,282.6141507491457,352.6841676092724,172.6829403069612,407.04467772479614,175.29986174933387,165.317551364732,57.27063637886884,84.01469248942257,30.266111029036672,324.12758763932663,14.45158423912577,41.749971374458404,91.52729721561033,40.59357712860112,47.24981040146311,79.92496037846938,10.59273543031209,1.2179580860554593,0.9214389793747422,0.9024303496134286,5.853591988159366,16.094491571751337,8.90584614047615,6.7585834009191705,6.7585834009191705,8.304244844053969,80.81489324721875,61.202511435630825,34.94719478867431,6.0515815395349755,11.436075434177653,17.53430830775565,20.42389373082748,26.347482339664527,8.606200576779365,12.828196694865065,6.139949738544274,1.6549118058498</t>
+          <t>26.41000528314367,4.784146385839009,50.553961630184446,51.35006941966825,1.338876163204955,1.7594353423943738,41.66161874249256,552.6564903042959,32.92970037665598,11.806137858078221,3.954996377327836,182.37658576441322,13.462658079332973,3.8875053954258116,132.51871785042246,41.1886047592809,44.67004700147301,13.140915986299055,7.929026468775817,5.358828114963549,175.77139743082063,87.07310509427444,31.84176004483261,346.3437031855027,26.134474774316573,2.2359841082049097,181.59792147881186,69.23091033377081,35.37739102126763,416.7808489258462,35.50565410515054,149.00406098930193,25.53151185108639,292.568066003213,80.09111358538928,34.89301648887374,44.84337107351443,315.51453012329057,31.776833720040194,195.48520442375846,0.019611618515110864,54.668603446610575,133.75400424675624,14.117214434716605,5.300927391448344,8.023931098717703,0.8691127015976078,0.28037947529547663,9.207126117665538,15.322162427638522,6.7585834009191705,13.56084049319578,42.67918740391483,2.5713723648926448,0.8548872337571174,50.10979837355765,34.94719478867431,28.305443465875282,38.3120468516971,50.61919057421116,47.16489655409354,3.3283411532899607,6.286068001131252,6.132096402169513,11.031012848937374,3.4586161268408278</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2458,11 +2458,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>-4.853126386208806</v>
+        <v>-6.317786712575508</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15.86484533359101,36.34214052692148,15.320901650504386,24.255407500548177,10.090750054617324,13.221378985987304,42.67560099878069,206.23582713245645,46.89894777520771,220.47250653164585,59.26230254329684,221.39188816311938,11.243605586920193,1.713807437951852,43.816294052902045,127.46327793062652,66.14565238330309,12.14290822744194,0.8900074955439067,13.384452743650984,84.01469248942257,308.8122947381376,216.80270160365524,467.7434254093612,146.90839610035954,246.3224064713823,123.09570937595399,126.2205442068202,282.6141507491457,352.6841676092724,172.6829403069612,407.04467772479614,175.29986174933387,165.317551364732,57.27063637886884,84.01469248942257,30.266111029036672,324.12758763932663,14.45158423912577,41.749971374458404,91.52729721561033,40.59357712860112,47.24981040146311,79.92496037846938,10.59273543031209,1.2179580860554593,0.9214389793747422,0.9024303496134286,5.853591988159366,16.094491571751337,8.90584614047615,6.7585834009191705,6.7585834009191705,8.304244844053969,80.81489324721875,61.202511435630825,34.94719478867431,6.0515815395349755,11.436075434177653,17.53430830775565,20.42389373082748,26.347482339664527,8.606200576779365,12.828196694865065,6.139949738544274,1.6549118058498</t>
+          <t>26.41000528314367,4.784146385839009,50.553961630184446,51.35006941966825,1.338876163204955,1.7594353423943738,41.66161874249256,552.6564903042959,32.92970037665598,11.806137858078221,3.954996377327836,182.37658576441322,13.462658079332973,3.8875053954258116,132.51871785042246,41.1886047592809,44.67004700147301,13.140915986299055,7.929026468775817,5.358828114963549,175.77139743082063,87.07310509427444,31.84176004483261,346.3437031855027,26.134474774316573,2.2359841082049097,181.59792147881186,69.23091033377081,35.37739102126763,416.7808489258462,35.50565410515054,149.00406098930193,25.53151185108639,292.568066003213,80.09111358538928,20.880694262847506,44.84337107351443,315.51453012329057,68.95380581041096,46.42947039992031,7.958558548987063,70.5736224028907,119.94573605394311,14.117214434716605,5.300927391448344,8.023931098717703,0.8691127015976078,0.28037947529547663,9.207126117665538,15.322162427638522,6.7585834009191705,13.56084049319578,42.67918740391483,2.5713723648926448,0.8548872337571174,50.10979837355765,34.94719478867431,28.305443465875282,38.3120468516971,50.61919057421116,47.16489655409354,3.3283411532899607,6.286068001131252,6.132096402169513,11.031012848937374,3.4586161268408278</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2471,11 +2471,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>-6.091883180614977</v>
+        <v>-6.775168358973645</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15.86484533359101,36.34214052692148,9.954921321991359,13.702235503131847,10.090750054617324,13.221378985987304,4.644936323967926,213.33171693468714,46.89894777520771,432.93373601644436,117.60171256929038,344.81257771862533,11.243605586920193,1.713807437951852,5.299162392270943,81.65632949067779,93.04281096146686,16.220668631477988,0.7154941206858325,2.0017219271557436,6.855844318399738,308.8122947381376,184.67585139736468,568.5430424544718,146.90839610035954,148.95731483701712,123.09570937595399,82.95434534377509,282.6141507491457,238.03692540300923,277.00276339652044,272.33774482192905,136.08334991286827,296.85880431632467,57.27063637886884,84.01469248942257,3.2411769432401294,433.31538775258053,16.106155469920832,41.749971374458404,91.52729721561033,46.075015564766424,43.664603545403466,79.92496037846938,11.981400364165312,1.3038739658084846,0.4432085919028644,0.9024303496134286,10.944570682307987,16.094491571751337,8.90584614047615,6.7585834009191705,10.593558526773888,8.304244844053969,80.81489324721875,86.96764856986711,21.38168723521047,6.0515815395349755,21.82289601064637,25.94553685860503,13.865226519310815,39.337512476629485,7.678602420760241,12.828196694865065,6.198427100476093,2.0089423645303084</t>
+          <t>43.57481008984285,23.897037108399367,22.444454773952426,24.255407500548177,10.55114691579316,10.94988802279714,55.812771901662565,130.2462617600637,53.21750908661978,417.71915496025844,3.367319303294597,354.56798323374346,6.7585834009191705,4.117429866264041,11.262284033237288,47.877437403209655,10.916181368240085,204.74860970967217,4.2623202046867785,7.739320627796387,15.230211745742826,505.1156329008741,44.849922811935805,70.69520891598323,195.34583976960107,36.747954200215865,62.44827157113572,509.13193024108165,57.27634900061284,343.5429459382562,0.8600981643645115,416.4640860697068,80.40693692893649,11.35035758605274,44.92387200649778,120.63807436421091,33.42104503782383,315.51453012329057,88.01045845131537,44.23470838303909,2.7163820332883803,32.44722737759192,17.26325895670325,107.00291130470463,3.6562091089990685,15.16359067734513,0.5461829993303907,0.43499969488111073,4.929884228570731,21.135129778643382,1.599386414851518,6.7585834009191705,2.6697072771452075,4.002536765765775,197.4990892439305,29.479247068349938,69.07409265598756,3.431684374717887,12.05943206792191,24.10754632382966,20.321480444909508,36.405479857510365,16.221354676447707,1.3014218106888635,3.2135581304395866,6.7585834009191705</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2484,11 +2484,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>-6.175734588487341</v>
+        <v>-6.805784015815333</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>35.25330351162232,25.420066600574494,13.807833754921065,46.28539210211825,6.7585834009191705,10.000683897119721,31.176765842520282,149.99610010139736,46.89894777520771,257.8203576058509,48.39924342302681,162.7195741543676,6.822952678276747,6.7585834009191705,53.18978876604946,167.68292240963916,51.02740527375966,100.40402579981847,9.515225833932908,6.7585834009191705,84.01469248942257,514.0235428375861,100.40402579981847,442.33700623085105,95.7610849733884,368.1702325789591,118.31924994700454,266.2236704789896,290.95491853858556,465.58924715385416,172.6829403069612,272.33115468409585,182.37658576441322,273.37641745672454,14.685334143219007,84.01469248942257,44.84337107351443,188.81034378587395,488.1615402958549,38.17023192810354,34.944556965917876,70.5736224028907,22.857636731609524,74.097785365391,6.7585834009191705,6.7585834009191705,0.5190731997727623,0.9024303496134286,4.929884228570731,14.894060786403676,6.7585834009191705,10.59273543031209,1.2179580860554593,6.7585834009191705,210.5812885890211,33.58089166670025,34.94719478867431,33.58089166670025,10.704840986010058,15.230798380174132,12.333181388538627,19.073559087978698,10.73266737637785,7.7360987720335705,5.8094366652553235,6.7585834009191705</t>
+          <t>24.809118641174802,45.78216022758797,22.568146776004824,24.255407500548177,4.1896744479353085,2.6414841812349557,69.69572165752622,130.2462617600637,46.89894777520771,223.62782635592004,48.39924342302681,221.7821325718657,10.697591705580853,0.831635887748323,11.262284033237288,78.01303808162544,42.4697700177014,337.3659023781316,4.2623202046867785,16.745183316501972,15.232649445709463,438.60755644602665,44.849922811935805,70.69520891598323,32.40289017666175,369.33939339332306,70.8040732748386,54.44163405917775,370.563754747831,60.893920690060156,453.29473090296636,27.78494225376866,182.37658576441322,239.03180078010345,87.68136913946489,101.93584462766005,44.84337107351443,179.42460800523105,347.20166978340455,31.542148988904867,28.094624972433877,32.44722737759192,84.41863003022884,87.47493150244102,2.160829291034198,11.193203901931001,1.2263436676287405,0.43499969488111073,4.929884228570731,14.958413270980516,1.6830506260644438,6.7585834009191705,4.748838769030488,2.035947340992194,179.93667657965747,52.51139585910695,69.07409265598756,3.431684374717887,12.05943206792191,0.1774064250486515,20.321480444909508,23.03510699883788,16.221354676447707,0.7905641559716957,6.7585834009191705,6.7585834009191705</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2497,11 +2497,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>-6.593095890607847</v>
+        <v>-7.004853523432987</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>24.809118641174802,28.2582006607538,33.394113627410576,16.466337112089224,6.7585834009191705,6.7585834009191705,62.839622680726485,149.99610010139736,29.425766773197992,201.6021425635028,48.86020160597532,221.39188816311938,6.520073499465089,6.7585834009191705,52.6452531600657,51.11938823203096,40.84185878402426,195.46221416219103,7.2601836529345425,8.594551289645272,84.01469248942257,222.39630223232683,90.63139770632552,449.1205744821289,13.840627500734044,158.46385452502778,274.86887349882676,304.2486053209648,165.73760446636297,354.4507536369641,247.43019892631705,272.33115468409585,68.07086085176742,71.24964940234592,66.31664222155128,84.01469248942257,120.30932490364953,188.81034378587395,170.90165177723048,16.26768477739841,34.944556965917876,70.5736224028907,129.3940953114266,100.13815064639437,18.00110713650346,4.787962664930429,0.058229307082543744,1.3969589073290123,4.237552234544849,12.708637455710834,6.7585834009191705,2.793518168319291,6.139949738544274,1.7161935045022199,281.12800139592343,59.92128280359042,112.55680316523623,33.58089166670025,2.8044936485904457,13.885508016496184,27.61376551087795,4.56503702315984,0.24171861659253105,8.896247730634403,4.891504517858715,6.7585834009191705</t>
+          <t>39.268261713321266,45.78216022758797,22.568146776004824,2.4786984142111463,20.056516218008266,26.383907477840935,55.812771901662565,211.01788600650565,56.997270277127114,223.62782635592004,48.39924342302681,307.8823671067553,8.752499305988641,15.298617125109239,11.262284033237288,24.915116464544237,37.10724661997721,204.74860970967217,4.2623202046867785,10.335605055744553,13.496018689132212,393.50774747845765,44.849922811935805,70.69520891598323,30.35841020263406,196.46788252107086,69.83201450653047,29.19151078316834,424.11547270563705,46.2317968493267,453.29473090296636,35.665393582612786,247.83782058276861,446.4193952386525,119.77886695392934,131.3761653228524,44.84337107351443,179.42460800523105,347.20166978340455,55.600618605499,52.39596207062338,0.23877778909873215,101.95224532935904,107.00291130470463,2.160829291034198,11.193203901931001,1.464801975926691,0.43499969488111073,7.214870134640714,14.958413270980516,3.0855490924046904,2.5713723648926448,2.542728865910718,1.7751965511857153,162.74915924677285,33.58089166670025,63.109183488910254,4.005483763818673,12.05943206792191,24.10754632382966,38.94862340110217,33.09254020344779,16.221354676447707,0.7905641559716957,8.129313191826299,6.7585834009191705</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2510,11 +2510,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>-6.852040015595315</v>
+        <v>-7.047491176506354</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>24.809118641174802,8.655667292387253,33.03893899122842,37.3757459455472,6.7585834009191705,10.115668078543084,45.924309390235386,149.99610010139736,46.89894777520771,230.53334989516514,89.81243217525528,182.37658576441322,11.243605586920193,1.713807437951852,43.816294052902045,127.46327793062652,66.14565238330309,12.14290822744194,0.8900074955439067,13.384452743650984,84.01469248942257,308.8122947381376,216.80270160365524,467.7434254093612,146.90839610035954,246.3224064713823,123.09570937595399,126.2205442068202,282.6141507491457,352.6841676092724,172.6829403069612,407.04467772479614,175.29986174933387,165.317551364732,57.27063637886884,84.01469248942257,46.705125882270416,259.60313231824097,330.6878306878307,41.749971374458404,34.944556965917876,70.5736224028907,59.692153001871596,38.29422414982758,3.7972210260837413,12.136309609634392,0.032385376267611746,1.1656323820506183,4.929884228570731,16.709093583745684,7.03917838844613,6.7585834009191705,9.292655188968281,6.7585834009191705,305.16375552167995,33.58089166670025,34.94719478867431,24.30406988527341,3.587313692669016,14.715752180739912,12.333181388538627,19.073559087978698,19.586380919779188,7.7360987720335705,7.03917838844613,9.292655188968281</t>
+          <t>4.38127944001331,45.78216022758797,37.18571380233075,18.92334968531565,10.94988802279714,8.21384749694395,45.924309390235386,130.2462617600637,60.73506584209305,622.1860518843687,159.31901941622246,143.00673727325145,10.588145562121229,3.336136566583331,88.1358971710767,106.08683844247548,28.362617565015434,6.7591985309578835,6.585025124365607,9.827672453455465,104.73692574446905,44.35742032900656,258.96406358510916,133.18367472569022,86.98956425282024,2.2359841082049097,181.59792147881186,69.23091033377081,122.62188404051517,389.4411885084851,35.50565410515054,149.00406098930193,25.53151185108639,292.568066003213,80.09111358538928,34.89301648887374,44.84337107351443,315.51453012329057,31.776833720040194,195.48520442375846,0.026650903516553106,102.0999080855732,182.7173005675227,422.5424356398108,1.3098834994378654,8.796739408793202,0.4510223991775007,0.9024303496134286,0.004751193833546584,11.071986213229353,15.931046807156312,3.539701963527189,6.7585834009191705,5.928776545222211,229.83665974222205,49.145529823308465,106.10756282820103,43.02522076711055,2.576809595676117,13.280137561472303,21.662036631854583,9.955876853535026,12.30320381340317,6.696735509574655,6.7585834009191705,7.66914804304478</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2523,11 +2523,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>-7.869042665305091</v>
+        <v>-7.140928088046442</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>24.809118641174802,8.309661551843158,22.568146776004824,35.805844627977,9.121570971490382,6.7585834009191705,45.924309390235386,77.51897375283417,26.976028563402043,172.6829403069612,48.39924342302681,354.42701475465043,10.59273543031209,1.2179580860554593,43.816294052902045,106.08683844247548,45.52547226401465,86.30371103231174,6.7585834009191705,6.7585834009191705,84.01469248942257,453.45364270871374,91.21374042296304,234.76823679663434,106.08683844247548,246.3224064713823,30.14130781725904,266.2236704789896,260.340366538962,271.214389550652,246.3549071966246,286.90415306680717,28.170742281878564,273.37641745672454,58.97172251524248,73.3181649145264,49.41461404008686,161.93474039746278,330.6878306878307,95.60809641608883,5.042749453664671,70.5736224028907,93.5308685371488,55.94889087900327,6.7585834009191705,6.769085079875938,1.043717365115723,1.5083004885280307,4.929884228570731,7.579112634935475,5.796554502986554,4.531825415764952,7.532377987800143,4.367843532515641,368.30637825934724,66.53756578777136,34.94719478867431,44.830806301014604,19.86452136451176,15.230798380174132,12.333181388538627,4.996961224193617,12.405040274547277,7.7360987720335705,6.7585834009191705,6.7585834009191705</t>
+          <t>43.57481008984285,23.897037108399367,22.568146776004824,24.255407500548177,11.07513590793465,10.374649805178352,93.43712833465968,317.55022679838254,2.255896482911869,168.03870618875075,4.945995152584616,201.58229442790676,4.2623202046867785,5.779198702274163,11.262284033237288,32.43504670509042,42.4697700177014,204.74860970967217,4.2623202046867785,12.559066421881173,12.533849908230781,318.55263745413595,44.849922811935805,70.69520891598323,25.02115430502808,362.90511002069866,123.09570937595399,54.44163405917775,128.4182455105871,56.55262339459598,847.3430538071015,26.580845656365554,182.37658576441322,239.03180078010345,17.9304755430271,84.01469248942257,75.8767675343466,243.06903877316657,210.1388206370203,55.600618605499,74.03161272378138,32.44722737759192,80.22219173908236,112.34640657747724,4.248046355507941,16.78311983369355,0.9024303496134286,0.38186786721846355,9.40961255082202,14.958413270980516,1.6830506260644438,6.7585834009191705,2.542728865910718,2.035947340992194,216.8341980749823,33.58089166670025,69.07409265598756,1.6316906323856792,12.05943206792191,24.10754632382966,7.645391328349098,19.073559087978698,3.913140635486854,0.9872102296603396,4.227491230736753,6.7585834009191705</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2536,11 +2536,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>-8.875521809509614</v>
+        <v>-7.390464807067931</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>18.233258892742672,27.213221398242467,12.749077169166302,2.6400289794432967,3.362703562326555,6.7585834009191705,85.86554224727553,149.99610010139736,144.34983159150798,172.6829403069612,96.0447648730402,284.04717613960486,1.1614907288211265,6.7585834009191705,17.173944918132424,106.08683844247548,59.73947857427783,100.40402579981847,6.7585834009191705,6.7585834009191705,84.01469248942257,273.45715473299646,191.59602668686423,347.38683922550734,106.08683844247548,167.22158896432404,183.7852642226233,266.2236704789896,149.99610010139736,271.214389550652,172.6829403069612,272.33115468409585,182.37658576441322,243.9112128673529,44.92387200649778,84.01469248942257,44.84337107351443,190.60858827975403,401.4309343586275,44.703153633016605,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,6.7585834009191705,6.7585834009191705,1.0842695677860266,0.9024303496134286,4.929884228570731,10.789934521779642,6.7585834009191705,12.704260701080782,14.192079705436724,6.100749997428718,239.01653502104344,46.38381094834184,33.59114542749077,73.67792982477809,11.459970281064813,7.325955223007839,12.333181388538627,35.66219101430774,15.693481959883021,10.992854762432373,11.602348100607728,6.7585834009191705</t>
+          <t>64.44368235882335,82.8311558154464,17.606998900439688,18.92334968531565,29.096019113959418,10.8930941515326,104.91026519569593,170.0019406208649,4.487849888774891,34.23886077562775,91.82245878430537,12.31206261704897,11.765464578582142,0.3231547247108502,89.41367731861574,79.43802541479826,15.570892867559763,55.60125822664,0.28317001990885937,6.518179275670625,46.54736685268359,26.377534246565816,148.12183532461754,26.947664044313928,106.08683844247548,7.624189731230026,237.16636898378022,500.47309361675724,521.9464080898487,197.86157933160172,104.1251551831278,247.95071905920798,13.925691385741931,445.4177454879818,83.90089529204928,17.983800226975884,53.0792419502923,306.03794870790483,269.65140022100184,28.702004259168902,50.01374384293209,49.8241960083461,30.386016491213777,7.674727083661451,13.28692447098856,56.913375360416424,0.19689176322946314,4.169666414107233,1.1351220905672812,0.5384542737474481,4.578043989029921,3.539701963527189,13.257088047984467,5.928776545222211,26.32605315806683,33.58089166670025,68.47741444043406,45.5894317332653,8.094896761447458,15.230798380174132,21.662036631854583,15.75831787999777,9.957407524580933,3.2291839998656644,12.624501131925651,0.5369094215093145</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2549,11 +2549,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>-9.087046673122218</v>
+        <v>-7.549883708359451</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>41.139114576166996,47.678188210560045,24.16012453521941,20.01828429459446,0.7960061898964004,3.0942196293740003,79.70841596295071,260.340366538962,149.61421464080837,172.6829403069612,50.98918616000964,259.1537903606004,4.3563707826792095,1.0439624712780842,12.915172874356385,206.06401713251313,42.4697700177014,68.161565052797,8.80602255026815,7.915767457263167,93.46071056256768,238.64131586621247,115.19009878800391,201.3509043887316,411.3852844370284,246.3224064713823,123.09570937595399,185.761280023643,79.5581625519325,388.5250886926519,243.11561716687947,294.57095422102566,182.65996768623262,273.37641745672454,73.74394574515354,196.03309335451223,44.91304997786726,361.29396806810917,298.5009820170478,28.282046669902133,34.944556965917876,70.5736224028907,44.22860883333776,74.097785365391,2.3013334388701154,9.89431816738774,1.3905768220938182,1.350680362907341,4.929884228570731,7.663998062541289,6.7585834009191705,9.022772424364058,7.532377987800143,12.54161780981613,55.1688611845529,33.58089166670025,43.29895148329336,44.46054617030914,15.887085577028321,13.342613289704902,8.926103134778673,6.391766096634034,12.340571549752635,21.983908974828115,4.891504517858715,6.7585834009191705</t>
+          <t>42.87319408525826,25.280743732758275,21.382558348126825,18.92334968531565,6.7585834009191705,14.550496312561478,85.78299053039446,170.0019406208649,5.85051679707882,172.6829403069612,90.4137700678956,182.37658576441322,6.7585834009191705,6.7585834009191705,43.816294052902045,106.08683844247548,42.4697700177014,51.590955038321,0.45498780184301924,6.7585834009191705,146.25430063204365,531.6425430826094,100.40402579981847,60.343454916422495,106.08683844247548,309.5417513812083,186.99612734272003,266.2236704789896,19.17777022234374,747.2536708846111,27.664508755900503,610.3381685412437,5.235847148194181,124.50912842634936,45.02784931942241,96.51895606539432,24.90816869207132,57.521933496401886,2.883548177098335,156.89733582297248,11.413609441819114,166.80625891340324,38.67211412668786,144.62233509391095,0.5652290933740395,8.37692203323078,2.127966038642687,1.5825951917109384,8.498166656328006,29.407243433634445,0.213522530218442,14.640102174755127,6.7585834009191705,14.460473350798187,251.40958876687117,33.58089166670025,57.87767256329671,70.82785159567219,6.772874593521949,15.230798380174132,10.299823174588504,9.955876853535026,3.7461973967718047,1.7681703773095834,8.439723229292037,7.66914804304478</t>
         </is>
       </c>
       <c r="C21" t="n">

</xml_diff>